<commit_message>
fix: report total QDPX project file counts
</commit_message>
<xml_diff>
--- a/reports/23071063-sq26-classification.xlsx
+++ b/reports/23071063-sq26-classification.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
@@ -535,7 +535,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
@@ -559,7 +559,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
@@ -583,7 +583,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">

</xml_diff>